<commit_message>
Added new parameter mapping
</commit_message>
<xml_diff>
--- a/Data/mvpf_component_mapping.xlsx
+++ b/Data/mvpf_component_mapping.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/td/PycharmProjects/CCJ/Data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{13BEA313-A8D3-694B-916A-22A561E94937}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6B5F196C-4EA6-7D4D-8BBD-155146AED92B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="760" windowWidth="29400" windowHeight="17480" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -1813,7 +1813,9 @@
       <c r="F11" s="6">
         <v>1</v>
       </c>
-      <c r="G11" s="6"/>
+      <c r="G11" s="9">
+        <v>0.25</v>
+      </c>
       <c r="H11" s="6">
         <v>1</v>
       </c>

</xml_diff>

<commit_message>
New layout with extra features for graphs and benchmarking added, with content review.
</commit_message>
<xml_diff>
--- a/Data/mvpf_component_mapping.xlsx
+++ b/Data/mvpf_component_mapping.xlsx
@@ -8,19 +8,20 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/td/PycharmProjects/CCJ/Data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6B5F196C-4EA6-7D4D-8BBD-155146AED92B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C21932F3-C4CA-324F-BF25-3B85D9BC70E7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="760" windowWidth="29400" windowHeight="17480" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="9020" yWindow="880" windowWidth="20380" windowHeight="17480" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet 1" sheetId="1" r:id="rId1"/>
+    <sheet name="Reviewed" sheetId="1" r:id="rId1"/>
+    <sheet name="Sheet 1 (2)" sheetId="2" r:id="rId2"/>
   </sheets>
   <calcPr calcId="0"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="41" uniqueCount="41">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="71" uniqueCount="45">
   <si>
     <t>mvpf_component_mapping</t>
   </si>
@@ -143,13 +144,25 @@
   </si>
   <si>
     <t>Assumption</t>
+  </si>
+  <si>
+    <t>1. Baseline</t>
+  </si>
+  <si>
+    <t>4. Most conservative</t>
+  </si>
+  <si>
+    <t>2.  Least conservative</t>
+  </si>
+  <si>
+    <t>NO</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="5">
+  <fonts count="7">
     <font>
       <sz val="10"/>
       <color indexed="8"/>
@@ -180,8 +193,21 @@
       <name val="JetBrains Mono"/>
       <family val="3"/>
     </font>
+    <font>
+      <sz val="10"/>
+      <color rgb="FFFF0000"/>
+      <name val="Helvetica Neue"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="10"/>
+      <color rgb="FFFF0000"/>
+      <name val="Helvetica Neue"/>
+      <family val="2"/>
+    </font>
   </fonts>
-  <fills count="4">
+  <fills count="10">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -198,6 +224,42 @@
       <patternFill patternType="solid">
         <fgColor indexed="12"/>
         <bgColor auto="1"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFF00"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="8" tint="0.39997558519241921"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="6" tint="0.39997558519241921"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4" tint="0.39997558519241921"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9" tint="0.39997558519241921"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5" tint="0.39997558519241921"/>
+        <bgColor indexed="64"/>
       </patternFill>
     </fill>
   </fills>
@@ -320,7 +382,7 @@
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="22">
+  <cellXfs count="36">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
@@ -372,19 +434,61 @@
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="49" fontId="3" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="49" fontId="3" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="6" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="7" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="7" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="7" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="7" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="7" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="7" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="7" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="8" borderId="7" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="49" fontId="0" fillId="9" borderId="7" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="49" fontId="6" fillId="3" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="8" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top"/>
     </xf>
   </cellXfs>
@@ -1517,6 +1621,380 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
+  <dimension ref="A1:J12"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="7.33203125" defaultRowHeight="20" customHeight="1"/>
+  <cols>
+    <col min="1" max="1" width="13" style="1" customWidth="1"/>
+    <col min="2" max="11" width="15.6640625" style="1" customWidth="1"/>
+    <col min="12" max="16384" width="7.33203125" style="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:10" ht="27.75" customHeight="1">
+      <c r="A1" s="32" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="32"/>
+      <c r="C1" s="32"/>
+      <c r="D1" s="32"/>
+      <c r="E1" s="32"/>
+      <c r="F1" s="32"/>
+      <c r="G1" s="32"/>
+      <c r="H1" s="32"/>
+      <c r="I1" s="32"/>
+      <c r="J1" s="32"/>
+    </row>
+    <row r="2" spans="1:10" ht="20.25" customHeight="1">
+      <c r="A2" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="B2" s="2" t="s">
+        <v>41</v>
+      </c>
+      <c r="C2" s="2" t="s">
+        <v>43</v>
+      </c>
+      <c r="D2" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="E2" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="F2" s="2" t="s">
+        <v>42</v>
+      </c>
+      <c r="G2" s="16" t="s">
+        <v>21</v>
+      </c>
+      <c r="H2" s="3">
+        <v>3</v>
+      </c>
+      <c r="I2" s="3" t="s">
+        <v>19</v>
+      </c>
+      <c r="J2" s="3" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="3" spans="1:10" s="14" customFormat="1" ht="81" customHeight="1">
+      <c r="A3" s="11" t="s">
+        <v>7</v>
+      </c>
+      <c r="B3" s="12" t="s">
+        <v>17</v>
+      </c>
+      <c r="C3" s="12" t="s">
+        <v>26</v>
+      </c>
+      <c r="D3" s="12" t="s">
+        <v>28</v>
+      </c>
+      <c r="E3" s="12" t="s">
+        <v>30</v>
+      </c>
+      <c r="F3" s="17" t="s">
+        <v>25</v>
+      </c>
+      <c r="G3" s="12" t="s">
+        <v>29</v>
+      </c>
+      <c r="H3" s="12" t="s">
+        <v>44</v>
+      </c>
+      <c r="I3" s="12" t="s">
+        <v>27</v>
+      </c>
+      <c r="J3" s="12" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="4" spans="1:10" ht="20" customHeight="1">
+      <c r="A4" s="7" t="s">
+        <v>8</v>
+      </c>
+      <c r="B4" s="9">
+        <v>0</v>
+      </c>
+      <c r="C4" s="9">
+        <v>0</v>
+      </c>
+      <c r="D4" s="9">
+        <v>0</v>
+      </c>
+      <c r="E4" s="9">
+        <v>0</v>
+      </c>
+      <c r="F4" s="22">
+        <v>1</v>
+      </c>
+      <c r="G4" s="23">
+        <v>1</v>
+      </c>
+      <c r="H4" s="25">
+        <v>1</v>
+      </c>
+      <c r="I4" s="25">
+        <v>1</v>
+      </c>
+      <c r="J4" s="26">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="5" spans="1:10" ht="20" customHeight="1">
+      <c r="A5" s="7" t="s">
+        <v>9</v>
+      </c>
+      <c r="B5" s="27">
+        <v>1</v>
+      </c>
+      <c r="C5" s="28">
+        <v>1</v>
+      </c>
+      <c r="D5" s="28">
+        <v>1</v>
+      </c>
+      <c r="E5" s="28">
+        <v>1</v>
+      </c>
+      <c r="F5" s="8">
+        <v>0</v>
+      </c>
+      <c r="G5" s="9">
+        <v>1</v>
+      </c>
+      <c r="H5" s="9">
+        <v>0</v>
+      </c>
+      <c r="I5" s="9">
+        <v>0</v>
+      </c>
+      <c r="J5" s="6">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="6" spans="1:10" ht="20" customHeight="1">
+      <c r="A6" s="7" t="s">
+        <v>10</v>
+      </c>
+      <c r="B6" s="9">
+        <v>1</v>
+      </c>
+      <c r="C6" s="9">
+        <v>1</v>
+      </c>
+      <c r="D6" s="6">
+        <v>1</v>
+      </c>
+      <c r="E6" s="6">
+        <v>0</v>
+      </c>
+      <c r="F6" s="8">
+        <v>1</v>
+      </c>
+      <c r="G6" s="6">
+        <v>0</v>
+      </c>
+      <c r="H6" s="9">
+        <v>1</v>
+      </c>
+      <c r="I6" s="6">
+        <v>0</v>
+      </c>
+      <c r="J6" s="6">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="7" spans="1:10" ht="20" customHeight="1">
+      <c r="A7" s="7" t="s">
+        <v>11</v>
+      </c>
+      <c r="B7" s="6"/>
+      <c r="C7" s="6"/>
+      <c r="D7" s="9">
+        <v>1</v>
+      </c>
+      <c r="E7" s="9">
+        <v>0</v>
+      </c>
+      <c r="F7" s="5"/>
+      <c r="G7" s="6">
+        <v>1</v>
+      </c>
+      <c r="H7" s="6"/>
+      <c r="I7" s="6"/>
+      <c r="J7" s="6"/>
+    </row>
+    <row r="8" spans="1:10" ht="20" customHeight="1">
+      <c r="A8" s="7" t="s">
+        <v>12</v>
+      </c>
+      <c r="B8" s="35">
+        <v>0</v>
+      </c>
+      <c r="C8" s="9">
+        <v>0</v>
+      </c>
+      <c r="D8" s="6"/>
+      <c r="E8" s="31" t="s">
+        <v>13</v>
+      </c>
+      <c r="F8" s="8">
+        <v>0</v>
+      </c>
+      <c r="G8" s="30">
+        <v>1</v>
+      </c>
+      <c r="H8" s="9">
+        <v>0</v>
+      </c>
+      <c r="I8" s="30">
+        <v>1</v>
+      </c>
+      <c r="J8" s="30">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="9" spans="1:10" ht="20" customHeight="1">
+      <c r="A9" s="7" t="s">
+        <v>18</v>
+      </c>
+      <c r="B9" s="27">
+        <v>0</v>
+      </c>
+      <c r="C9" s="28">
+        <v>1</v>
+      </c>
+      <c r="D9" s="28">
+        <v>0.25</v>
+      </c>
+      <c r="E9" s="29">
+        <v>1</v>
+      </c>
+      <c r="F9" s="22">
+        <v>0</v>
+      </c>
+      <c r="G9" s="24">
+        <v>0</v>
+      </c>
+      <c r="H9" s="25">
+        <v>0.25</v>
+      </c>
+      <c r="I9" s="26">
+        <v>1</v>
+      </c>
+      <c r="J9" s="26">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="10" spans="1:10" ht="20" customHeight="1">
+      <c r="A10" s="7" t="s">
+        <v>14</v>
+      </c>
+      <c r="B10" s="9">
+        <v>1</v>
+      </c>
+      <c r="C10" s="9">
+        <v>1</v>
+      </c>
+      <c r="D10" s="6">
+        <v>1</v>
+      </c>
+      <c r="E10" s="6">
+        <v>1</v>
+      </c>
+      <c r="F10" s="8">
+        <v>1</v>
+      </c>
+      <c r="G10" s="6">
+        <v>1</v>
+      </c>
+      <c r="H10" s="9">
+        <v>1</v>
+      </c>
+      <c r="I10" s="6">
+        <v>1</v>
+      </c>
+      <c r="J10" s="6">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="11" spans="1:10" ht="20" customHeight="1">
+      <c r="A11" s="34" t="s">
+        <v>15</v>
+      </c>
+      <c r="B11" s="9">
+        <v>0</v>
+      </c>
+      <c r="C11" s="9">
+        <v>0</v>
+      </c>
+      <c r="D11" s="33">
+        <v>1</v>
+      </c>
+      <c r="E11" s="33">
+        <v>1</v>
+      </c>
+      <c r="F11" s="8">
+        <v>0</v>
+      </c>
+      <c r="G11" s="33">
+        <v>1</v>
+      </c>
+      <c r="H11" s="9">
+        <v>0</v>
+      </c>
+      <c r="I11" s="6">
+        <v>0</v>
+      </c>
+      <c r="J11" s="33">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="12" spans="1:10" ht="20" customHeight="1">
+      <c r="A12" s="7" t="s">
+        <v>16</v>
+      </c>
+      <c r="B12" s="9">
+        <v>0</v>
+      </c>
+      <c r="C12" s="9">
+        <v>0</v>
+      </c>
+      <c r="D12" s="6">
+        <v>0</v>
+      </c>
+      <c r="E12" s="6">
+        <v>0</v>
+      </c>
+      <c r="F12" s="8">
+        <v>0</v>
+      </c>
+      <c r="G12" s="6">
+        <v>0</v>
+      </c>
+      <c r="H12" s="9">
+        <v>0</v>
+      </c>
+      <c r="I12" s="6">
+        <v>0</v>
+      </c>
+      <c r="J12" s="6">
+        <v>0</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="1" right="1" top="1" bottom="1" header="0.25" footer="0.25"/>
+  <pageSetup orientation="portrait"/>
+  <headerFooter>
+    <oddFooter>&amp;C&amp;"Helvetica Neue,Regular"&amp;12&amp;K000000&amp;P</oddFooter>
+  </headerFooter>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FC389DCE-C1ED-D248-8F2B-2D9E4D002CFF}">
+  <sheetPr>
+    <pageSetUpPr fitToPage="1"/>
+  </sheetPr>
   <dimension ref="A1:J14"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="21" defaultRowHeight="20" customHeight="1"/>
   <cols>
@@ -1526,18 +2004,18 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:10" ht="27.75" customHeight="1">
-      <c r="A1" s="17" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="17"/>
-      <c r="C1" s="17"/>
-      <c r="D1" s="17"/>
-      <c r="E1" s="17"/>
-      <c r="F1" s="17"/>
-      <c r="G1" s="17"/>
-      <c r="H1" s="17"/>
-      <c r="I1" s="17"/>
-      <c r="J1" s="17"/>
+      <c r="A1" s="21" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="21"/>
+      <c r="C1" s="21"/>
+      <c r="D1" s="21"/>
+      <c r="E1" s="21"/>
+      <c r="F1" s="21"/>
+      <c r="G1" s="21"/>
+      <c r="H1" s="21"/>
+      <c r="I1" s="21"/>
+      <c r="J1" s="21"/>
     </row>
     <row r="2" spans="1:10" ht="20.25" customHeight="1">
       <c r="A2" s="2" t="s">
@@ -1578,7 +2056,7 @@
       <c r="B3" s="12" t="s">
         <v>17</v>
       </c>
-      <c r="C3" s="18" t="s">
+      <c r="C3" s="17" t="s">
         <v>25</v>
       </c>
       <c r="D3" s="12" t="s">
@@ -1620,31 +2098,31 @@
       <c r="I4" s="6"/>
       <c r="J4" s="6"/>
     </row>
-    <row r="5" spans="1:10" s="20" customFormat="1" ht="63" customHeight="1">
-      <c r="A5" s="21" t="s">
+    <row r="5" spans="1:10" s="19" customFormat="1" ht="63" customHeight="1">
+      <c r="A5" s="20" t="s">
         <v>32</v>
       </c>
       <c r="B5" s="15"/>
-      <c r="C5" s="19" t="s">
+      <c r="C5" s="18" t="s">
         <v>33</v>
       </c>
-      <c r="D5" s="19" t="s">
+      <c r="D5" s="18" t="s">
         <v>34</v>
       </c>
       <c r="E5" s="15"/>
-      <c r="F5" s="19" t="s">
+      <c r="F5" s="18" t="s">
         <v>35</v>
       </c>
-      <c r="G5" s="19" t="s">
+      <c r="G5" s="18" t="s">
         <v>36</v>
       </c>
-      <c r="H5" s="19" t="s">
+      <c r="H5" s="18" t="s">
         <v>37</v>
       </c>
-      <c r="I5" s="19" t="s">
+      <c r="I5" s="18" t="s">
         <v>38</v>
       </c>
-      <c r="J5" s="19" t="s">
+      <c r="J5" s="18" t="s">
         <v>39</v>
       </c>
     </row>

</xml_diff>